<commit_message>
Now calculated g from the ball on incline experiment + created figure to show fitting for acceleration
</commit_message>
<xml_diff>
--- a/BallOnIncline/Ball_data/BallOnIncline_Group1_data.xlsx
+++ b/BallOnIncline/Ball_data/BallOnIncline_Group1_data.xlsx
@@ -4,19 +4,19 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="hældning_længder"/>
-    <sheet r:id="rId2" sheetId="2" name="Trigonometriske målinger"/>
-    <sheet r:id="rId3" sheetId="3" name="Goniometer vinkelmål"/>
+    <sheet r:id="rId2" sheetId="2" name="trigonometriske_målinger"/>
+    <sheet r:id="rId3" sheetId="3" name="goniometer_vinkelmål"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="57">
   <si>
     <t>Vinkelmålinger med goniometer i grader.</t>
   </si>
@@ -78,13 +78,19 @@
     <t>Højde</t>
   </si>
   <si>
-    <t>Usikkerhed</t>
+    <t>u_højde</t>
   </si>
   <si>
     <t>Længde</t>
   </si>
   <si>
+    <t>u_længde</t>
+  </si>
+  <si>
     <t>Hypotenuse</t>
+  </si>
+  <si>
+    <t>u_hypo</t>
   </si>
   <si>
     <t>0.2</t>
@@ -188,7 +194,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -200,6 +206,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -247,8 +259,8 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -569,140 +581,140 @@
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="2" t="s">
+      <c r="F3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>33</v>
+      <c r="G5" s="2" t="s">
+        <v>52</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>34</v>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="2" t="s">
+        <v>53</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>35</v>
+      <c r="B6" s="2" t="s">
+        <v>54</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>36</v>
+      <c r="C6" s="2" t="s">
+        <v>55</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F5" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
@@ -9664,7 +9676,7 @@
     <col min="7" max="7" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="14.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="32.25">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -9678,16 +9690,16 @@
         <v>21</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="14.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="21">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
@@ -9707,21 +9719,21 @@
         <v>93.1</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="14.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="5">
-        <v>22275</v>
+        <v>22.275</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3" s="5">
-        <v>90150</v>
+        <v>90.15</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>17</v>
@@ -18712,12 +18724,12 @@
   <cols>
     <col min="1" max="1" style="3" width="33.71928571428572" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="3" width="8.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="10.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="3" width="20.290714285714284" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="3" width="22.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="14.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="27">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>